<commit_message>
Modification du schéma de la BDD + Programmation classes
- Modification UML
</commit_message>
<xml_diff>
--- a/Documentation/HoferL-JournalPlanif-M5.xlsx
+++ b/Documentation/HoferL-JournalPlanif-M5.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Journal" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="SommeParJours" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Plannification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="PlanificationExemple" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Journal" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="SommeParJours" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Plannification" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="PlanificationExemple" sheetId="4" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$B$2:$H$30</definedName>
@@ -21,8 +21,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>date</t>
   </si>
@@ -169,6 +191,12 @@
   </si>
   <si>
     <t xml:space="preserve">Finalisation de la maquette + test</t>
+  </si>
+  <si>
+    <t>03.03.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programmation des classes + test SQLite</t>
   </si>
   <si>
     <t>Phases</t>
@@ -194,9 +222,6 @@
   </si>
   <si>
     <t>02.03.2026</t>
-  </si>
-  <si>
-    <t>03.03.2026</t>
   </si>
   <si>
     <t>16.03.2026</t>
@@ -2301,7 +2326,7 @@
             <c:strRef>
               <c:f>SommeParJours!$A$2:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>20.01.2026</c:v>
                 </c:pt>
@@ -2331,6 +2356,15 @@
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>12.02.2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>13.02.2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>24.02.2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>03.03.2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2370,6 +2404,15 @@
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0.08333333333333333</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.0625</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.125</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2692,8 +2735,8 @@
   </c:chart>
   <c:spPr bwMode="auto">
     <a:xfrm rot="0">
-      <a:off x="0" y="0"/>
-      <a:ext cx="0" cy="0"/>
+      <a:off x="1973108" y="70845"/>
+      <a:ext cx="5882350" cy="3850639"/>
     </a:xfrm>
     <a:prstGeom prst="rect">
       <a:avLst/>
@@ -3391,15 +3434,15 @@
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>512609</xdr:colOff>
+      <xdr:colOff>68108</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>70846</xdr:rowOff>
+      <xdr:rowOff>70845</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>383626</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>701125</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>9886</xdr:rowOff>
+      <xdr:rowOff>9885</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3409,8 +3452,8 @@
         </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm rot="0">
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
+        <a:off x="1973108" y="70845"/>
+        <a:ext cx="5882350" cy="3850639"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3424,8 +3467,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E25">
-  <autoFilter ref="B2:E25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E26">
+  <autoFilter ref="B2:E26"/>
   <tableColumns count="4">
     <tableColumn id="1" name="date" dataDxfId="0"/>
     <tableColumn id="2" name="Temps" dataDxfId="1"/>
@@ -3986,7 +4029,7 @@
       </c>
       <c r="I3" s="9">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.065217391304347824</v>
+        <v>0.056074766355140186</v>
       </c>
       <c r="J3" s="10"/>
     </row>
@@ -4012,7 +4055,7 @@
       </c>
       <c r="I4" s="9">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.065217391304347824</v>
+        <v>0.056074766355140186</v>
       </c>
     </row>
     <row r="5" ht="28.5">
@@ -4037,7 +4080,7 @@
       </c>
       <c r="I5" s="9">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.13043478260869565</v>
+        <v>0.11214953271028037</v>
       </c>
     </row>
     <row r="6">
@@ -4058,11 +4101,11 @@
       </c>
       <c r="H6" s="8">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>11</v>
+        <v>15.499999999999998</v>
       </c>
       <c r="I6" s="9">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.2391304347826087</v>
+        <v>0.28971962616822428</v>
       </c>
     </row>
     <row r="7">
@@ -4087,7 +4130,7 @@
       </c>
       <c r="I7" s="9">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.4565217391304347</v>
+        <v>0.39252336448598124</v>
       </c>
     </row>
     <row r="8" ht="28.5">
@@ -4108,11 +4151,11 @@
       </c>
       <c r="H8" s="8">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I8" s="9">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.043478260869565216</v>
+        <v>0.093457943925233641</v>
       </c>
     </row>
     <row r="9">
@@ -4183,7 +4226,7 @@
       </c>
       <c r="H11" s="8">
         <f>SUM(H3:H10)</f>
-        <v>46</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="12">
@@ -4371,24 +4414,32 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C25" s="4">
         <v>0.125</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="3"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="6"/>
+      <c r="B26" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="3"/>
@@ -4718,7 +4769,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{00770051-00AC-442C-B38D-008B00050008}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00D900E8-00A9-48EE-A1ED-003400B10084}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$10</xm:f>
           </x14:formula1>
@@ -4732,7 +4783,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" customWidth="1" min="3" max="3" style="17" width="5.6640625"/>
     <col bestFit="1" customWidth="1" min="4" max="4" width="12.21875"/>
@@ -4750,8 +4801,8 @@
       <c r="C1"/>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="str">
-        <f t="array" ref="A2:A13">_xlfn.UNIQUE(Journal[date])</f>
+      <c r="A2" s="18" t="str" cm="1">
+        <f t="array" ref="A2:A14">_xlfn.UNIQUE(Journal[date])</f>
         <v>20.01.2026</v>
       </c>
       <c r="B2" s="19">
@@ -4882,7 +4933,14 @@
       <c r="C13"/>
     </row>
     <row r="14">
-      <c r="A14" s="18"/>
+      <c r="A14" s="18" t="str">
+        <f/>
+        <v>03.03.2026</v>
+      </c>
+      <c r="B14" s="19">
+        <f>SUMIF(Journal[date],SommeParJours!A14,Journal[Temps])</f>
+        <v>0.125</v>
+      </c>
       <c r="C14"/>
     </row>
     <row r="15">
@@ -6391,7 +6449,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="4.33203125"/>
     <col bestFit="1" min="3" max="3" width="35.77734375"/>
@@ -6408,16 +6466,16 @@
   <sheetData>
     <row r="1" s="24" customFormat="1" ht="66.599999999999994" customHeight="1">
       <c r="B1" s="25" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D1" s="27" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F1" s="28" t="s">
         <v>11</v>
@@ -6426,7 +6484,7 @@
         <v>17</v>
       </c>
       <c r="H1" s="30" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I1" s="27" t="s">
         <v>22</v>
@@ -6435,85 +6493,85 @@
         <v>37</v>
       </c>
       <c r="K1" s="27" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="L1" s="31" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="M1" s="27" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="N1" s="29" t="s">
         <v>47</v>
       </c>
       <c r="O1" s="30" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="P1" s="27" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="Q1" s="27" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="R1" s="27" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S1" s="27" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="T1" s="27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="U1" s="27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="V1" s="29" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W1" s="32" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="X1" s="27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Y1" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Z1" s="29" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AA1" s="33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AB1" s="34" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AC1" s="34" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AD1" s="31" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AE1" s="35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AF1" s="36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AG1" s="37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AH1" s="37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AI1" s="37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AJ1" s="37" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AK1" s="34" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AL1" s="38"/>
       <c r="AM1" s="38"/>
@@ -6609,7 +6667,7 @@
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="39"/>
       <c r="C4" s="40" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D4" s="41"/>
       <c r="E4" s="41"/>
@@ -6765,7 +6823,7 @@
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="39"/>
       <c r="C8" s="40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D8" s="55"/>
       <c r="E8" s="55"/>
@@ -6843,7 +6901,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="39"/>
       <c r="C10" s="40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D10" s="41"/>
       <c r="E10" s="41"/>
@@ -6921,7 +6979,7 @@
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="39"/>
       <c r="C12" s="40" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D12" s="41"/>
       <c r="E12" s="41"/>
@@ -6998,10 +7056,10 @@
     </row>
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="56" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C14" s="57" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D14" s="55"/>
       <c r="E14" s="55"/>
@@ -7079,7 +7137,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="56"/>
       <c r="C16" s="57" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D16" s="55"/>
       <c r="E16" s="55"/>
@@ -7154,13 +7212,13 @@
       <c r="AJ17" s="59"/>
       <c r="AK17" s="59"/>
       <c r="AN17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="56"/>
       <c r="C18" s="57" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D18" s="55"/>
       <c r="E18" s="55"/>
@@ -7238,7 +7296,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="56"/>
       <c r="C20" s="57" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D20" s="59"/>
       <c r="E20" s="59"/>
@@ -7316,7 +7374,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="56"/>
       <c r="C22" s="57" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D22" s="59"/>
       <c r="E22" s="59"/>
@@ -7394,7 +7452,7 @@
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="56"/>
       <c r="C24" s="57" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D24" s="59"/>
       <c r="E24" s="59"/>
@@ -7471,10 +7529,10 @@
     </row>
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" s="40" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D26" s="41"/>
       <c r="E26" s="41"/>
@@ -7552,7 +7610,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="39"/>
       <c r="C28" s="40" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D28" s="41"/>
       <c r="E28" s="41"/>
@@ -7630,7 +7688,7 @@
     <row r="30" ht="12" customHeight="1">
       <c r="B30" s="39"/>
       <c r="C30" s="40" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D30" s="41"/>
       <c r="E30" s="41"/>
@@ -7708,7 +7766,7 @@
     <row r="32" ht="12" customHeight="1">
       <c r="B32" s="39"/>
       <c r="C32" s="40" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D32" s="41"/>
       <c r="E32" s="41"/>
@@ -7785,10 +7843,10 @@
     </row>
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="56" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C34" s="66" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D34" s="59"/>
       <c r="E34" s="59"/>
@@ -7866,7 +7924,7 @@
     <row r="36" ht="12" customHeight="1">
       <c r="B36" s="56"/>
       <c r="C36" s="66" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D36" s="59"/>
       <c r="E36" s="59"/>
@@ -7944,7 +8002,7 @@
     <row r="38" ht="12" customHeight="1">
       <c r="B38" s="56"/>
       <c r="C38" s="66" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D38" s="59"/>
       <c r="E38" s="59"/>
@@ -8022,7 +8080,7 @@
     <row r="40" ht="12" customHeight="1">
       <c r="B40" s="56"/>
       <c r="C40" s="66" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D40" s="59"/>
       <c r="E40" s="59"/>
@@ -8102,7 +8160,7 @@
         <v>21</v>
       </c>
       <c r="C42" s="68" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D42" s="41"/>
       <c r="E42" s="41"/>
@@ -8180,7 +8238,7 @@
     <row r="44" ht="12" customHeight="1">
       <c r="B44" s="39"/>
       <c r="C44" s="68" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D44" s="41"/>
       <c r="E44" s="41"/>
@@ -8257,7 +8315,7 @@
     </row>
     <row r="46" ht="12" customHeight="1">
       <c r="B46" s="56" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C46" s="57" t="s">
         <v>24</v>
@@ -8335,14 +8393,14 @@
       <c r="AJ47" s="59"/>
       <c r="AK47" s="59"/>
       <c r="AN47" s="69" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AO47" s="55"/>
     </row>
     <row r="48" ht="12" customHeight="1">
       <c r="B48" s="56"/>
       <c r="C48" s="57" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D48" s="59"/>
       <c r="E48" s="59"/>
@@ -8379,7 +8437,7 @@
       <c r="AJ48" s="59"/>
       <c r="AK48" s="70"/>
       <c r="AN48" s="69" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AO48" s="54"/>
     </row>
@@ -8421,28 +8479,19 @@
       <c r="AJ49" s="59"/>
       <c r="AK49" s="59"/>
       <c r="AN49" s="69" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AO49" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="B34:B41"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="B26:B33"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="B2:B13"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C12:C13"/>
     <mergeCell ref="B14:B25"/>
     <mergeCell ref="C14:C15"/>
     <mergeCell ref="C16:C17"/>
@@ -8450,13 +8499,22 @@
     <mergeCell ref="C20:C21"/>
     <mergeCell ref="C22:C23"/>
     <mergeCell ref="C24:C25"/>
-    <mergeCell ref="B2:B13"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="B26:B33"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="B34:B41"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="C48:C49"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -8490,37 +8548,37 @@
     </row>
     <row r="2" ht="56.399999999999999" customHeight="1">
       <c r="B2" s="72" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C2" s="73" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" s="74" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E2" s="75" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F2" s="76" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G2" s="76"/>
       <c r="H2" s="76"/>
       <c r="I2" s="75"/>
       <c r="J2" s="76" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K2" s="76"/>
       <c r="L2" s="76"/>
       <c r="M2" s="75"/>
       <c r="N2" s="76" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O2" s="76"/>
       <c r="P2" s="76"/>
       <c r="Q2" s="75"/>
       <c r="R2" s="76" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="S2" s="77"/>
       <c r="AD2" s="21"/>
@@ -8529,7 +8587,7 @@
       <c r="B3" s="78"/>
       <c r="C3" s="79"/>
       <c r="D3" s="80" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" s="81">
         <v>4</v>
@@ -8577,15 +8635,15 @@
         <v>2</v>
       </c>
       <c r="U3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="85" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C4" s="73" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D4" s="86"/>
       <c r="E4" s="87"/>
@@ -8604,7 +8662,7 @@
       <c r="R4" s="90"/>
       <c r="S4" s="91"/>
       <c r="U4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -8630,7 +8688,7 @@
     <row r="6" ht="12" customHeight="1">
       <c r="B6" s="85"/>
       <c r="C6" s="100" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D6" s="101"/>
       <c r="E6" s="102"/>
@@ -8649,7 +8707,7 @@
       <c r="R6" s="106"/>
       <c r="S6" s="107"/>
       <c r="U6" s="108" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="V6" s="108"/>
     </row>
@@ -8673,13 +8731,13 @@
       <c r="R7" s="98"/>
       <c r="S7" s="99"/>
       <c r="U7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="85"/>
       <c r="C8" s="100" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D8" s="101"/>
       <c r="E8" s="102"/>
@@ -8698,7 +8756,7 @@
       <c r="R8" s="106"/>
       <c r="S8" s="107"/>
       <c r="U8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -8724,7 +8782,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="85"/>
       <c r="C10" s="100" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D10" s="101"/>
       <c r="E10" s="102"/>
@@ -8765,10 +8823,10 @@
     </row>
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="72" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C12" s="73" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D12" s="86"/>
       <c r="E12" s="87"/>
@@ -8810,7 +8868,7 @@
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="85"/>
       <c r="C14" s="100" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D14" s="119"/>
       <c r="E14" s="102"/>
@@ -8852,7 +8910,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="85"/>
       <c r="C16" s="100" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D16" s="101"/>
       <c r="E16" s="102"/>
@@ -8893,10 +8951,10 @@
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="74" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C18" s="73" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D18" s="86"/>
       <c r="E18" s="87"/>
@@ -8938,7 +8996,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="85"/>
       <c r="C20" s="100" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D20" s="101"/>
       <c r="E20" s="102"/>
@@ -8980,7 +9038,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="85"/>
       <c r="C22" s="100" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D22" s="101"/>
       <c r="E22" s="102"/>
@@ -9021,10 +9079,10 @@
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="74" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C24" s="73" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D24" s="86"/>
       <c r="E24" s="87"/>
@@ -9066,7 +9124,7 @@
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="85"/>
       <c r="C26" s="100" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D26" s="101"/>
       <c r="E26" s="102"/>
@@ -9108,7 +9166,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="85"/>
       <c r="C28" s="100" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D28" s="101"/>
       <c r="E28" s="102"/>
@@ -9152,7 +9210,7 @@
         <v>12</v>
       </c>
       <c r="C30" s="132" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D30" s="86"/>
       <c r="E30" s="133"/>
@@ -9236,7 +9294,7 @@
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="138"/>
       <c r="C34" s="92" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D34" s="124"/>
       <c r="E34" s="152"/>
@@ -9256,7 +9314,7 @@
       <c r="S34" s="156"/>
       <c r="U34" s="157"/>
       <c r="V34" s="158" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" ht="13.800000000000001" customHeight="1">
@@ -9280,7 +9338,7 @@
       <c r="S35" s="116"/>
       <c r="U35" s="165"/>
       <c r="V35" s="166" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modification de la documentation
.docx
</commit_message>
<xml_diff>
--- a/Documentation/HoferL-JournalPlanif-M5.xlsx
+++ b/Documentation/HoferL-JournalPlanif-M5.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="1" state="visible" r:id="rId2"/>
@@ -2039,66 +2039,11 @@
           <c:cat>
             <c:strRef>
               <c:f>Journal!$G$3:$G$10</c:f>
-              <c:strCache>
-                <c:ptCount val="8"/>
-                <c:pt idx="0">
-                  <c:v>Cours</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Plannification</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Recherche</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Maquettage</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Documentation</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Programmation</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Tests</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Présentation</c:v>
-                </c:pt>
-              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Journal!$I$3:$I$10</c:f>
-              <c:numCache>
-                <c:formatCode>0%</c:formatCode>
-                <c:ptCount val="8"/>
-                <c:pt idx="0">
-                  <c:v>0.06521739130434782</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.06521739130434782</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.13043478260869565</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.2391304347826087</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.4565217391304347</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.043478260869565216</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
+              <c:f>Journal!$H$3:$H$10</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -4769,7 +4714,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{00D900E8-00A9-48EE-A1ED-003400B10084}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00CC0040-003C-41BA-B267-00AB00D30038}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$10</xm:f>
           </x14:formula1>
@@ -6796,7 +6741,7 @@
       <c r="L7" s="45"/>
       <c r="M7" s="41"/>
       <c r="N7" s="46"/>
-      <c r="O7" s="47"/>
+      <c r="O7" s="53"/>
       <c r="P7" s="41"/>
       <c r="Q7" s="41"/>
       <c r="R7" s="41"/>
@@ -6864,17 +6809,17 @@
       <c r="B9" s="39"/>
       <c r="C9" s="40"/>
       <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="49"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="51"/>
       <c r="G9" s="46"/>
       <c r="H9" s="47"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="41"/>
+      <c r="I9" s="54"/>
+      <c r="J9" s="54"/>
       <c r="K9" s="41"/>
       <c r="L9" s="45"/>
-      <c r="M9" s="41"/>
+      <c r="M9" s="54"/>
       <c r="N9" s="46"/>
-      <c r="O9" s="47"/>
+      <c r="O9" s="53"/>
       <c r="P9" s="41"/>
       <c r="Q9" s="41"/>
       <c r="R9" s="41"/>
@@ -7896,9 +7841,9 @@
       <c r="K35" s="67"/>
       <c r="L35" s="45"/>
       <c r="M35" s="59"/>
-      <c r="N35" s="60"/>
+      <c r="N35" s="52"/>
       <c r="O35" s="58"/>
-      <c r="P35" s="59"/>
+      <c r="P35" s="54"/>
       <c r="Q35" s="59"/>
       <c r="R35" s="59"/>
       <c r="S35" s="59"/>
@@ -7976,7 +7921,7 @@
       <c r="M37" s="59"/>
       <c r="N37" s="60"/>
       <c r="O37" s="58"/>
-      <c r="P37" s="59"/>
+      <c r="P37" s="54"/>
       <c r="Q37" s="59"/>
       <c r="R37" s="59"/>
       <c r="S37" s="59"/>

</xml_diff>

<commit_message>
Ajout de différentes documentations
</commit_message>
<xml_diff>
--- a/Documentation/HoferL-JournalPlanif-M5.xlsx
+++ b/Documentation/HoferL-JournalPlanif-M5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\Desktop\ScholarLog\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC831C6-9A90-44DB-AD49-EAEEEAF2F259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459BF26C-B436-48F0-99EA-6CF5AC0F8218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="162">
   <si>
     <t>date</t>
   </si>
@@ -553,6 +553,15 @@
   </si>
   <si>
     <t>&lt;-- A jour avec la BDD</t>
+  </si>
+  <si>
+    <t>Documentation des fichiers MVVM + Documentation du repertoire intérrction avec la BDD.</t>
+  </si>
+  <si>
+    <t>Implémentation correction de la séparation en MVVM.</t>
+  </si>
+  <si>
+    <t>Recherche de pratique de programmation sur les MVVM.</t>
   </si>
 </sst>
 </file>
@@ -565,7 +574,7 @@
     <numFmt numFmtId="166" formatCode="0.0&quot; H&quot;;@"/>
     <numFmt numFmtId="167" formatCode="0&quot;H&quot;"/>
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="170" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="169" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -1768,6 +1777,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
@@ -1846,10 +1859,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2252,16 +2261,16 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>31.5</c:v>
+                  <c:v>33.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>40.5</c:v>
+                  <c:v>41.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3677,8 +3686,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Journal" displayName="Journal" ref="B2:E44">
-  <autoFilter ref="B2:E44" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Journal" displayName="Journal" ref="B2:E47">
+  <autoFilter ref="B2:E47" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="date" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Temps" dataDxfId="3"/>
@@ -3959,7 +3968,7 @@
       </c>
       <c r="I3" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>2.9411764705882353E-2</v>
+        <v>2.8301886792452831E-2</v>
       </c>
       <c r="J3" s="11" t="str" cm="1">
         <f t="array" ref="J3:J9">_xlfn._xlws.FILTER(G3:G10,H3:H10&gt;0)</f>
@@ -3992,7 +4001,7 @@
       </c>
       <c r="I4" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>2.9411764705882353E-2</v>
+        <v>2.8301886792452831E-2</v>
       </c>
       <c r="J4" s="3" t="str">
         <v>Plannification</v>
@@ -4019,17 +4028,17 @@
       </c>
       <c r="H5" s="9">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>5.8823529411764705E-2</v>
+        <v>6.6037735849056603E-2</v>
       </c>
       <c r="J5" s="3" t="str">
         <v>Recherche</v>
       </c>
       <c r="K5" s="12">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.3">
@@ -4054,7 +4063,7 @@
       </c>
       <c r="I6" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.16666666666666666</v>
+        <v>0.16037735849056603</v>
       </c>
       <c r="J6" s="3" t="str">
         <v>Maquettage</v>
@@ -4081,17 +4090,17 @@
       </c>
       <c r="H7" s="9">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>31.5</v>
+        <v>33.5</v>
       </c>
       <c r="I7" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.30882352941176472</v>
+        <v>0.31603773584905659</v>
       </c>
       <c r="J7" s="3" t="str">
         <v>Documentation</v>
       </c>
       <c r="K7" s="12">
-        <v>31.5</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="8" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
@@ -4112,17 +4121,17 @@
       </c>
       <c r="H8" s="9">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>40.5</v>
+        <v>41.5</v>
       </c>
       <c r="I8" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.39705882352941174</v>
+        <v>0.39150943396226418</v>
       </c>
       <c r="J8" s="3" t="str">
         <v>Programmation</v>
       </c>
       <c r="K8" s="12">
-        <v>40.5</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
@@ -4147,7 +4156,7 @@
       </c>
       <c r="I9" s="10">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>9.8039215686274508E-3</v>
+        <v>9.433962264150943E-3</v>
       </c>
       <c r="J9" s="3" t="str">
         <v>Tests</v>
@@ -4201,7 +4210,7 @@
       </c>
       <c r="H11" s="9">
         <f>SUM(H3:H10)</f>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
@@ -4599,9 +4608,9 @@
       <c r="E39" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H39" s="171"/>
-      <c r="I39" s="170"/>
-      <c r="J39" s="172"/>
+      <c r="H39" s="145"/>
+      <c r="I39" s="144"/>
+      <c r="J39" s="146"/>
     </row>
     <row r="40" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B40" s="4">
@@ -4677,22 +4686,46 @@
       </c>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B45" s="4"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="7"/>
+      <c r="B45" s="4">
+        <v>46100</v>
+      </c>
+      <c r="C45" s="5">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B46" s="4"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="7"/>
-    </row>
-    <row r="47" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B47" s="4"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="7"/>
+      <c r="B46" s="4">
+        <v>46100</v>
+      </c>
+      <c r="C46" s="5">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B47" s="4">
+        <v>46100</v>
+      </c>
+      <c r="C47" s="5">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="48" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B48" s="16"/>
@@ -4934,7 +4967,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="str" cm="1">
-        <f t="array" ref="A2:A24">_xlfn.UNIQUE(Journal[date])</f>
+        <f t="array" ref="A2:A25">_xlfn.UNIQUE(Journal[date])</f>
         <v>20.01.2026</v>
       </c>
       <c r="B2" s="19">
@@ -5140,7 +5173,9 @@
       <c r="C24"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="18"/>
+      <c r="A25" s="18">
+        <v>46100</v>
+      </c>
       <c r="C25"/>
       <c r="F25" s="20"/>
     </row>
@@ -6741,10 +6776,10 @@
       <c r="AU1" s="39"/>
     </row>
     <row r="2" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="148" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="149" t="s">
+      <c r="C2" s="153" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="40"/>
@@ -6783,8 +6818,8 @@
       <c r="AK2" s="40"/>
     </row>
     <row r="3" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="144"/>
-      <c r="C3" s="149"/>
+      <c r="B3" s="148"/>
+      <c r="C3" s="153"/>
       <c r="D3" s="40"/>
       <c r="E3" s="40"/>
       <c r="F3" s="48"/>
@@ -6821,8 +6856,8 @@
       <c r="AK3" s="40"/>
     </row>
     <row r="4" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="144"/>
-      <c r="C4" s="149" t="s">
+      <c r="B4" s="148"/>
+      <c r="C4" s="153" t="s">
         <v>89</v>
       </c>
       <c r="D4" s="40"/>
@@ -6861,8 +6896,8 @@
       <c r="AK4" s="40"/>
     </row>
     <row r="5" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="144"/>
-      <c r="C5" s="149"/>
+      <c r="B5" s="148"/>
+      <c r="C5" s="153"/>
       <c r="D5" s="40"/>
       <c r="E5" s="40"/>
       <c r="F5" s="50"/>
@@ -6899,8 +6934,8 @@
       <c r="AK5" s="40"/>
     </row>
     <row r="6" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="144"/>
-      <c r="C6" s="149" t="s">
+      <c r="B6" s="148"/>
+      <c r="C6" s="153" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="40"/>
@@ -6939,8 +6974,8 @@
       <c r="AK6" s="54"/>
     </row>
     <row r="7" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="144"/>
-      <c r="C7" s="149"/>
+      <c r="B7" s="148"/>
+      <c r="C7" s="153"/>
       <c r="D7" s="40"/>
       <c r="E7" s="40"/>
       <c r="F7" s="50"/>
@@ -6977,8 +7012,8 @@
       <c r="AK7" s="40"/>
     </row>
     <row r="8" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="144"/>
-      <c r="C8" s="149" t="s">
+      <c r="B8" s="148"/>
+      <c r="C8" s="153" t="s">
         <v>90</v>
       </c>
       <c r="D8" s="54"/>
@@ -7017,8 +7052,8 @@
       <c r="AK8" s="54"/>
     </row>
     <row r="9" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="144"/>
-      <c r="C9" s="149"/>
+      <c r="B9" s="148"/>
+      <c r="C9" s="153"/>
       <c r="D9" s="40"/>
       <c r="E9" s="53"/>
       <c r="F9" s="50"/>
@@ -7055,8 +7090,8 @@
       <c r="AK9" s="40"/>
     </row>
     <row r="10" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="144"/>
-      <c r="C10" s="149" t="s">
+      <c r="B10" s="148"/>
+      <c r="C10" s="153" t="s">
         <v>91</v>
       </c>
       <c r="D10" s="40"/>
@@ -7095,8 +7130,8 @@
       <c r="AK10" s="40"/>
     </row>
     <row r="11" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="144"/>
-      <c r="C11" s="149"/>
+      <c r="B11" s="148"/>
+      <c r="C11" s="153"/>
       <c r="D11" s="40"/>
       <c r="E11" s="40"/>
       <c r="F11" s="48"/>
@@ -7133,8 +7168,8 @@
       <c r="AK11" s="40"/>
     </row>
     <row r="12" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="144"/>
-      <c r="C12" s="149" t="s">
+      <c r="B12" s="148"/>
+      <c r="C12" s="153" t="s">
         <v>92</v>
       </c>
       <c r="D12" s="40"/>
@@ -7173,8 +7208,8 @@
       <c r="AK12" s="54"/>
     </row>
     <row r="13" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="144"/>
-      <c r="C13" s="149"/>
+      <c r="B13" s="148"/>
+      <c r="C13" s="153"/>
       <c r="D13" s="40"/>
       <c r="E13" s="40"/>
       <c r="F13" s="48"/>
@@ -7211,10 +7246,10 @@
       <c r="AK13" s="40"/>
     </row>
     <row r="14" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="146" t="s">
+      <c r="B14" s="150" t="s">
         <v>93</v>
       </c>
-      <c r="C14" s="147" t="s">
+      <c r="C14" s="151" t="s">
         <v>94</v>
       </c>
       <c r="D14" s="54"/>
@@ -7253,8 +7288,8 @@
       <c r="AK14" s="56"/>
     </row>
     <row r="15" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="146"/>
-      <c r="C15" s="147"/>
+      <c r="B15" s="150"/>
+      <c r="C15" s="151"/>
       <c r="D15" s="56"/>
       <c r="E15" s="53"/>
       <c r="F15" s="50"/>
@@ -7291,8 +7326,8 @@
       <c r="AK15" s="56"/>
     </row>
     <row r="16" spans="2:47" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="146"/>
-      <c r="C16" s="147" t="s">
+      <c r="B16" s="150"/>
+      <c r="C16" s="151" t="s">
         <v>95</v>
       </c>
       <c r="D16" s="54"/>
@@ -7331,8 +7366,8 @@
       <c r="AK16" s="56"/>
     </row>
     <row r="17" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="146"/>
-      <c r="C17" s="147"/>
+      <c r="B17" s="150"/>
+      <c r="C17" s="151"/>
       <c r="D17" s="58"/>
       <c r="E17" s="53"/>
       <c r="F17" s="59"/>
@@ -7372,8 +7407,8 @@
       </c>
     </row>
     <row r="18" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="146"/>
-      <c r="C18" s="147" t="s">
+      <c r="B18" s="150"/>
+      <c r="C18" s="151" t="s">
         <v>97</v>
       </c>
       <c r="D18" s="54"/>
@@ -7412,8 +7447,8 @@
       <c r="AK18" s="56"/>
     </row>
     <row r="19" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="146"/>
-      <c r="C19" s="147"/>
+      <c r="B19" s="150"/>
+      <c r="C19" s="151"/>
       <c r="D19" s="56"/>
       <c r="E19" s="53"/>
       <c r="F19" s="60"/>
@@ -7450,8 +7485,8 @@
       <c r="AK19" s="56"/>
     </row>
     <row r="20" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="146"/>
-      <c r="C20" s="147" t="s">
+      <c r="B20" s="150"/>
+      <c r="C20" s="151" t="s">
         <v>98</v>
       </c>
       <c r="D20" s="56"/>
@@ -7490,8 +7525,8 @@
       <c r="AK20" s="56"/>
     </row>
     <row r="21" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="146"/>
-      <c r="C21" s="147"/>
+      <c r="B21" s="150"/>
+      <c r="C21" s="151"/>
       <c r="D21" s="56"/>
       <c r="E21" s="56"/>
       <c r="F21" s="59"/>
@@ -7528,8 +7563,8 @@
       <c r="AK21" s="56"/>
     </row>
     <row r="22" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="146"/>
-      <c r="C22" s="147" t="s">
+      <c r="B22" s="150"/>
+      <c r="C22" s="151" t="s">
         <v>99</v>
       </c>
       <c r="D22" s="56"/>
@@ -7568,8 +7603,8 @@
       <c r="AK22" s="56"/>
     </row>
     <row r="23" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="146"/>
-      <c r="C23" s="147"/>
+      <c r="B23" s="150"/>
+      <c r="C23" s="151"/>
       <c r="D23" s="56"/>
       <c r="E23" s="56"/>
       <c r="F23" s="59"/>
@@ -7606,8 +7641,8 @@
       <c r="AK23" s="56"/>
     </row>
     <row r="24" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="146"/>
-      <c r="C24" s="147" t="s">
+      <c r="B24" s="150"/>
+      <c r="C24" s="151" t="s">
         <v>100</v>
       </c>
       <c r="D24" s="56"/>
@@ -7646,8 +7681,8 @@
       <c r="AK24" s="56"/>
     </row>
     <row r="25" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="146"/>
-      <c r="C25" s="147"/>
+      <c r="B25" s="150"/>
+      <c r="C25" s="151"/>
       <c r="D25" s="56"/>
       <c r="E25" s="56"/>
       <c r="F25" s="59"/>
@@ -7684,10 +7719,10 @@
       <c r="AK25" s="56"/>
     </row>
     <row r="26" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="144" t="s">
+      <c r="B26" s="148" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="149" t="s">
+      <c r="C26" s="153" t="s">
         <v>102</v>
       </c>
       <c r="D26" s="40"/>
@@ -7726,8 +7761,8 @@
       <c r="AK26" s="40"/>
     </row>
     <row r="27" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="144"/>
-      <c r="C27" s="149"/>
+      <c r="B27" s="148"/>
+      <c r="C27" s="153"/>
       <c r="D27" s="40"/>
       <c r="E27" s="40"/>
       <c r="F27" s="48"/>
@@ -7764,8 +7799,8 @@
       <c r="AK27" s="40"/>
     </row>
     <row r="28" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="144"/>
-      <c r="C28" s="149" t="s">
+      <c r="B28" s="148"/>
+      <c r="C28" s="153" t="s">
         <v>103</v>
       </c>
       <c r="D28" s="40"/>
@@ -7804,8 +7839,8 @@
       <c r="AK28" s="40"/>
     </row>
     <row r="29" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="144"/>
-      <c r="C29" s="149"/>
+      <c r="B29" s="148"/>
+      <c r="C29" s="153"/>
       <c r="D29" s="40"/>
       <c r="E29" s="40"/>
       <c r="F29" s="48"/>
@@ -7842,8 +7877,8 @@
       <c r="AK29" s="40"/>
     </row>
     <row r="30" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="144"/>
-      <c r="C30" s="149" t="s">
+      <c r="B30" s="148"/>
+      <c r="C30" s="153" t="s">
         <v>104</v>
       </c>
       <c r="D30" s="40"/>
@@ -7882,8 +7917,8 @@
       <c r="AK30" s="40"/>
     </row>
     <row r="31" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="144"/>
-      <c r="C31" s="149"/>
+      <c r="B31" s="148"/>
+      <c r="C31" s="153"/>
       <c r="D31" s="40"/>
       <c r="E31" s="40"/>
       <c r="F31" s="50"/>
@@ -7920,8 +7955,8 @@
       <c r="AK31" s="40"/>
     </row>
     <row r="32" spans="2:40" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="144"/>
-      <c r="C32" s="149" t="s">
+      <c r="B32" s="148"/>
+      <c r="C32" s="153" t="s">
         <v>105</v>
       </c>
       <c r="D32" s="40"/>
@@ -7960,8 +7995,8 @@
       <c r="AK32" s="40"/>
     </row>
     <row r="33" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="144"/>
-      <c r="C33" s="149"/>
+      <c r="B33" s="148"/>
+      <c r="C33" s="153"/>
       <c r="D33" s="40"/>
       <c r="E33" s="40"/>
       <c r="F33" s="48"/>
@@ -7998,10 +8033,10 @@
       <c r="AK33" s="40"/>
     </row>
     <row r="34" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="146" t="s">
+      <c r="B34" s="150" t="s">
         <v>106</v>
       </c>
-      <c r="C34" s="148" t="s">
+      <c r="C34" s="152" t="s">
         <v>107</v>
       </c>
       <c r="D34" s="56"/>
@@ -8040,8 +8075,8 @@
       <c r="AK34" s="56"/>
     </row>
     <row r="35" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="146"/>
-      <c r="C35" s="148"/>
+      <c r="B35" s="150"/>
+      <c r="C35" s="152"/>
       <c r="D35" s="56"/>
       <c r="E35" s="56"/>
       <c r="F35" s="59"/>
@@ -8056,8 +8091,8 @@
       <c r="O35" s="55"/>
       <c r="P35" s="53"/>
       <c r="Q35" s="56"/>
-      <c r="R35" s="173"/>
-      <c r="S35" s="173"/>
+      <c r="R35" s="147"/>
+      <c r="S35" s="147"/>
       <c r="T35" s="56"/>
       <c r="U35" s="56"/>
       <c r="V35" s="57"/>
@@ -8078,8 +8113,8 @@
       <c r="AK35" s="56"/>
     </row>
     <row r="36" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="146"/>
-      <c r="C36" s="148" t="s">
+      <c r="B36" s="150"/>
+      <c r="C36" s="152" t="s">
         <v>108</v>
       </c>
       <c r="D36" s="56"/>
@@ -8118,8 +8153,8 @@
       <c r="AK36" s="56"/>
     </row>
     <row r="37" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="146"/>
-      <c r="C37" s="148"/>
+      <c r="B37" s="150"/>
+      <c r="C37" s="152"/>
       <c r="D37" s="56"/>
       <c r="E37" s="56"/>
       <c r="F37" s="59"/>
@@ -8134,8 +8169,8 @@
       <c r="O37" s="55"/>
       <c r="P37" s="53"/>
       <c r="Q37" s="56"/>
-      <c r="R37" s="173"/>
-      <c r="S37" s="173"/>
+      <c r="R37" s="147"/>
+      <c r="S37" s="147"/>
       <c r="T37" s="56"/>
       <c r="U37" s="56"/>
       <c r="V37" s="57"/>
@@ -8156,8 +8191,8 @@
       <c r="AK37" s="56"/>
     </row>
     <row r="38" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="146"/>
-      <c r="C38" s="148" t="s">
+      <c r="B38" s="150"/>
+      <c r="C38" s="152" t="s">
         <v>109</v>
       </c>
       <c r="D38" s="56"/>
@@ -8196,8 +8231,8 @@
       <c r="AK38" s="56"/>
     </row>
     <row r="39" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="146"/>
-      <c r="C39" s="148"/>
+      <c r="B39" s="150"/>
+      <c r="C39" s="152"/>
       <c r="D39" s="56"/>
       <c r="E39" s="56"/>
       <c r="F39" s="59"/>
@@ -8234,8 +8269,8 @@
       <c r="AK39" s="56"/>
     </row>
     <row r="40" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="146"/>
-      <c r="C40" s="148" t="s">
+      <c r="B40" s="150"/>
+      <c r="C40" s="152" t="s">
         <v>110</v>
       </c>
       <c r="D40" s="56"/>
@@ -8274,8 +8309,8 @@
       <c r="AK40" s="56"/>
     </row>
     <row r="41" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="146"/>
-      <c r="C41" s="148"/>
+      <c r="B41" s="150"/>
+      <c r="C41" s="152"/>
       <c r="D41" s="56"/>
       <c r="E41" s="56"/>
       <c r="F41" s="59"/>
@@ -8312,10 +8347,10 @@
       <c r="AK41" s="56"/>
     </row>
     <row r="42" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="144" t="s">
+      <c r="B42" s="148" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="145" t="s">
+      <c r="C42" s="149" t="s">
         <v>111</v>
       </c>
       <c r="D42" s="40"/>
@@ -8354,8 +8389,8 @@
       <c r="AK42" s="40"/>
     </row>
     <row r="43" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="144"/>
-      <c r="C43" s="145"/>
+      <c r="B43" s="148"/>
+      <c r="C43" s="149"/>
       <c r="D43" s="40"/>
       <c r="E43" s="40"/>
       <c r="F43" s="48"/>
@@ -8392,8 +8427,8 @@
       <c r="AK43" s="40"/>
     </row>
     <row r="44" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="144"/>
-      <c r="C44" s="145" t="s">
+      <c r="B44" s="148"/>
+      <c r="C44" s="149" t="s">
         <v>112</v>
       </c>
       <c r="D44" s="40"/>
@@ -8432,8 +8467,8 @@
       <c r="AK44" s="40"/>
     </row>
     <row r="45" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="144"/>
-      <c r="C45" s="145"/>
+      <c r="B45" s="148"/>
+      <c r="C45" s="149"/>
       <c r="D45" s="40"/>
       <c r="E45" s="40"/>
       <c r="F45" s="48"/>
@@ -8470,10 +8505,10 @@
       <c r="AK45" s="40"/>
     </row>
     <row r="46" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="146" t="s">
+      <c r="B46" s="150" t="s">
         <v>113</v>
       </c>
-      <c r="C46" s="147" t="s">
+      <c r="C46" s="151" t="s">
         <v>24</v>
       </c>
       <c r="D46" s="56"/>
@@ -8512,8 +8547,8 @@
       <c r="AK46" s="56"/>
     </row>
     <row r="47" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="146"/>
-      <c r="C47" s="147"/>
+      <c r="B47" s="150"/>
+      <c r="C47" s="151"/>
       <c r="D47" s="56"/>
       <c r="E47" s="56"/>
       <c r="F47" s="59"/>
@@ -8554,8 +8589,8 @@
       <c r="AO47" s="54"/>
     </row>
     <row r="48" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="146"/>
-      <c r="C48" s="147" t="s">
+      <c r="B48" s="150"/>
+      <c r="C48" s="151" t="s">
         <v>115</v>
       </c>
       <c r="D48" s="56"/>
@@ -8598,8 +8633,8 @@
       <c r="AO48" s="53"/>
     </row>
     <row r="49" spans="2:41" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="146"/>
-      <c r="C49" s="147"/>
+      <c r="B49" s="150"/>
+      <c r="C49" s="151"/>
       <c r="D49" s="56"/>
       <c r="E49" s="56"/>
       <c r="F49" s="59"/>
@@ -8700,10 +8735,10 @@
       <c r="B1" s="66"/>
     </row>
     <row r="2" spans="2:30" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="159" t="s">
+      <c r="B2" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="154" t="s">
+      <c r="C2" s="158" t="s">
         <v>62</v>
       </c>
       <c r="D2" s="67" t="s">
@@ -8712,33 +8747,33 @@
       <c r="E2" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="150" t="s">
+      <c r="F2" s="154" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="150"/>
-      <c r="H2" s="150"/>
-      <c r="I2" s="162"/>
-      <c r="J2" s="150" t="s">
+      <c r="G2" s="154"/>
+      <c r="H2" s="154"/>
+      <c r="I2" s="166"/>
+      <c r="J2" s="154" t="s">
         <v>121</v>
       </c>
-      <c r="K2" s="150"/>
-      <c r="L2" s="150"/>
-      <c r="M2" s="162"/>
-      <c r="N2" s="150" t="s">
+      <c r="K2" s="154"/>
+      <c r="L2" s="154"/>
+      <c r="M2" s="166"/>
+      <c r="N2" s="154" t="s">
         <v>122</v>
       </c>
-      <c r="O2" s="150"/>
-      <c r="P2" s="150"/>
-      <c r="Q2" s="162"/>
-      <c r="R2" s="150" t="s">
+      <c r="O2" s="154"/>
+      <c r="P2" s="154"/>
+      <c r="Q2" s="166"/>
+      <c r="R2" s="154" t="s">
         <v>123</v>
       </c>
-      <c r="S2" s="151"/>
+      <c r="S2" s="155"/>
       <c r="AD2" s="22"/>
     </row>
     <row r="3" spans="2:30" x14ac:dyDescent="0.3">
-      <c r="B3" s="160"/>
-      <c r="C3" s="161"/>
+      <c r="B3" s="164"/>
+      <c r="C3" s="165"/>
       <c r="D3" s="69" t="s">
         <v>124</v>
       </c>
@@ -8792,10 +8827,10 @@
       </c>
     </row>
     <row r="4" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="152" t="s">
+      <c r="B4" s="156" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="154" t="s">
+      <c r="C4" s="158" t="s">
         <v>127</v>
       </c>
       <c r="D4" s="74"/>
@@ -8819,8 +8854,8 @@
       </c>
     </row>
     <row r="5" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="152"/>
-      <c r="C5" s="155"/>
+      <c r="B5" s="156"/>
+      <c r="C5" s="159"/>
       <c r="D5" s="80"/>
       <c r="E5" s="81"/>
       <c r="F5" s="82"/>
@@ -8839,8 +8874,8 @@
       <c r="S5" s="86"/>
     </row>
     <row r="6" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="152"/>
-      <c r="C6" s="156" t="s">
+      <c r="B6" s="156"/>
+      <c r="C6" s="160" t="s">
         <v>129</v>
       </c>
       <c r="D6" s="87"/>
@@ -8859,14 +8894,14 @@
       <c r="Q6" s="88"/>
       <c r="R6" s="92"/>
       <c r="S6" s="93"/>
-      <c r="U6" s="157" t="s">
+      <c r="U6" s="161" t="s">
         <v>130</v>
       </c>
-      <c r="V6" s="157"/>
+      <c r="V6" s="161"/>
     </row>
     <row r="7" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="152"/>
-      <c r="C7" s="155"/>
+      <c r="B7" s="156"/>
+      <c r="C7" s="159"/>
       <c r="D7" s="80"/>
       <c r="E7" s="81"/>
       <c r="F7" s="85"/>
@@ -8888,8 +8923,8 @@
       </c>
     </row>
     <row r="8" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="152"/>
-      <c r="C8" s="156" t="s">
+      <c r="B8" s="156"/>
+      <c r="C8" s="160" t="s">
         <v>132</v>
       </c>
       <c r="D8" s="87"/>
@@ -8913,8 +8948,8 @@
       </c>
     </row>
     <row r="9" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="152"/>
-      <c r="C9" s="155"/>
+      <c r="B9" s="156"/>
+      <c r="C9" s="159"/>
       <c r="D9" s="80"/>
       <c r="E9" s="81"/>
       <c r="F9" s="85"/>
@@ -8933,8 +8968,8 @@
       <c r="S9" s="86"/>
     </row>
     <row r="10" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="152"/>
-      <c r="C10" s="156" t="s">
+      <c r="B10" s="156"/>
+      <c r="C10" s="160" t="s">
         <v>134</v>
       </c>
       <c r="D10" s="87"/>
@@ -8955,8 +8990,8 @@
       <c r="S10" s="93"/>
     </row>
     <row r="11" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="153"/>
-      <c r="C11" s="158"/>
+      <c r="B11" s="157"/>
+      <c r="C11" s="162"/>
       <c r="D11" s="94"/>
       <c r="E11" s="95"/>
       <c r="F11" s="96"/>
@@ -8975,10 +9010,10 @@
       <c r="S11" s="99"/>
     </row>
     <row r="12" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="159" t="s">
+      <c r="B12" s="163" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="154" t="s">
+      <c r="C12" s="158" t="s">
         <v>136</v>
       </c>
       <c r="D12" s="74"/>
@@ -8999,8 +9034,8 @@
       <c r="S12" s="79"/>
     </row>
     <row r="13" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="152"/>
-      <c r="C13" s="155"/>
+      <c r="B13" s="156"/>
+      <c r="C13" s="159"/>
       <c r="D13" s="80"/>
       <c r="E13" s="81"/>
       <c r="F13" s="85"/>
@@ -9019,8 +9054,8 @@
       <c r="S13" s="86"/>
     </row>
     <row r="14" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="152"/>
-      <c r="C14" s="156" t="s">
+      <c r="B14" s="156"/>
+      <c r="C14" s="160" t="s">
         <v>137</v>
       </c>
       <c r="D14" s="102"/>
@@ -9041,8 +9076,8 @@
       <c r="S14" s="93"/>
     </row>
     <row r="15" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="152"/>
-      <c r="C15" s="155"/>
+      <c r="B15" s="156"/>
+      <c r="C15" s="159"/>
       <c r="D15" s="80"/>
       <c r="E15" s="81"/>
       <c r="F15" s="85"/>
@@ -9061,8 +9096,8 @@
       <c r="S15" s="86"/>
     </row>
     <row r="16" spans="2:30" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="152"/>
-      <c r="C16" s="156" t="s">
+      <c r="B16" s="156"/>
+      <c r="C16" s="160" t="s">
         <v>138</v>
       </c>
       <c r="D16" s="87"/>
@@ -9083,8 +9118,8 @@
       <c r="S16" s="93"/>
     </row>
     <row r="17" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="153"/>
-      <c r="C17" s="158"/>
+      <c r="B17" s="157"/>
+      <c r="C17" s="162"/>
       <c r="D17" s="94"/>
       <c r="E17" s="95"/>
       <c r="F17" s="96"/>
@@ -9103,10 +9138,10 @@
       <c r="S17" s="99"/>
     </row>
     <row r="18" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="163" t="s">
+      <c r="B18" s="167" t="s">
         <v>139</v>
       </c>
-      <c r="C18" s="154" t="s">
+      <c r="C18" s="158" t="s">
         <v>140</v>
       </c>
       <c r="D18" s="74"/>
@@ -9127,8 +9162,8 @@
       <c r="S18" s="79"/>
     </row>
     <row r="19" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="152"/>
-      <c r="C19" s="155"/>
+      <c r="B19" s="156"/>
+      <c r="C19" s="159"/>
       <c r="D19" s="80"/>
       <c r="E19" s="81"/>
       <c r="F19" s="85"/>
@@ -9147,8 +9182,8 @@
       <c r="S19" s="86"/>
     </row>
     <row r="20" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="152"/>
-      <c r="C20" s="156" t="s">
+      <c r="B20" s="156"/>
+      <c r="C20" s="160" t="s">
         <v>141</v>
       </c>
       <c r="D20" s="87"/>
@@ -9169,8 +9204,8 @@
       <c r="S20" s="93"/>
     </row>
     <row r="21" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="152"/>
-      <c r="C21" s="155"/>
+      <c r="B21" s="156"/>
+      <c r="C21" s="159"/>
       <c r="D21" s="80"/>
       <c r="E21" s="81"/>
       <c r="F21" s="85"/>
@@ -9189,8 +9224,8 @@
       <c r="S21" s="86"/>
     </row>
     <row r="22" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="152"/>
-      <c r="C22" s="156" t="s">
+      <c r="B22" s="156"/>
+      <c r="C22" s="160" t="s">
         <v>142</v>
       </c>
       <c r="D22" s="87"/>
@@ -9211,8 +9246,8 @@
       <c r="S22" s="93"/>
     </row>
     <row r="23" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="153"/>
-      <c r="C23" s="158"/>
+      <c r="B23" s="157"/>
+      <c r="C23" s="162"/>
       <c r="D23" s="94"/>
       <c r="E23" s="95"/>
       <c r="F23" s="96"/>
@@ -9231,10 +9266,10 @@
       <c r="S23" s="99"/>
     </row>
     <row r="24" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="163" t="s">
+      <c r="B24" s="167" t="s">
         <v>143</v>
       </c>
-      <c r="C24" s="154" t="s">
+      <c r="C24" s="158" t="s">
         <v>144</v>
       </c>
       <c r="D24" s="74"/>
@@ -9255,8 +9290,8 @@
       <c r="S24" s="79"/>
     </row>
     <row r="25" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="152"/>
-      <c r="C25" s="155"/>
+      <c r="B25" s="156"/>
+      <c r="C25" s="159"/>
       <c r="D25" s="80"/>
       <c r="E25" s="81"/>
       <c r="F25" s="85"/>
@@ -9275,8 +9310,8 @@
       <c r="S25" s="86"/>
     </row>
     <row r="26" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="152"/>
-      <c r="C26" s="156" t="s">
+      <c r="B26" s="156"/>
+      <c r="C26" s="160" t="s">
         <v>145</v>
       </c>
       <c r="D26" s="87"/>
@@ -9297,8 +9332,8 @@
       <c r="S26" s="93"/>
     </row>
     <row r="27" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="152"/>
-      <c r="C27" s="155"/>
+      <c r="B27" s="156"/>
+      <c r="C27" s="159"/>
       <c r="D27" s="80"/>
       <c r="E27" s="81"/>
       <c r="F27" s="85"/>
@@ -9317,8 +9352,8 @@
       <c r="S27" s="86"/>
     </row>
     <row r="28" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="152"/>
-      <c r="C28" s="156" t="s">
+      <c r="B28" s="156"/>
+      <c r="C28" s="160" t="s">
         <v>146</v>
       </c>
       <c r="D28" s="87"/>
@@ -9339,8 +9374,8 @@
       <c r="S28" s="93"/>
     </row>
     <row r="29" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="152"/>
-      <c r="C29" s="161"/>
+      <c r="B29" s="156"/>
+      <c r="C29" s="165"/>
       <c r="D29" s="107"/>
       <c r="E29" s="108"/>
       <c r="F29" s="109"/>
@@ -9359,10 +9394,10 @@
       <c r="S29" s="113"/>
     </row>
     <row r="30" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="164" t="s">
+      <c r="B30" s="168" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="167" t="s">
+      <c r="C30" s="171" t="s">
         <v>90</v>
       </c>
       <c r="D30" s="74"/>
@@ -9383,8 +9418,8 @@
       <c r="S30" s="118"/>
     </row>
     <row r="31" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="165"/>
-      <c r="C31" s="168"/>
+      <c r="B31" s="169"/>
+      <c r="C31" s="172"/>
       <c r="D31" s="80"/>
       <c r="E31" s="119"/>
       <c r="F31" s="120"/>
@@ -9403,8 +9438,8 @@
       <c r="S31" s="86"/>
     </row>
     <row r="32" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="165"/>
-      <c r="C32" s="168" t="s">
+      <c r="B32" s="169"/>
+      <c r="C32" s="172" t="s">
         <v>12</v>
       </c>
       <c r="D32" s="87"/>
@@ -9425,8 +9460,8 @@
       <c r="S32" s="128"/>
     </row>
     <row r="33" spans="2:22" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="165"/>
-      <c r="C33" s="168"/>
+      <c r="B33" s="169"/>
+      <c r="C33" s="172"/>
       <c r="D33" s="80"/>
       <c r="E33" s="119"/>
       <c r="F33" s="123"/>
@@ -9445,8 +9480,8 @@
       <c r="S33" s="86"/>
     </row>
     <row r="34" spans="2:22" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="165"/>
-      <c r="C34" s="155" t="s">
+      <c r="B34" s="169"/>
+      <c r="C34" s="159" t="s">
         <v>147</v>
       </c>
       <c r="D34" s="107"/>
@@ -9471,8 +9506,8 @@
       </c>
     </row>
     <row r="35" spans="2:22" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="166"/>
-      <c r="C35" s="169"/>
+      <c r="B35" s="170"/>
+      <c r="C35" s="173"/>
       <c r="D35" s="94"/>
       <c r="E35" s="138"/>
       <c r="F35" s="139"/>

</xml_diff>

<commit_message>
Suppression de code dupliqué
</commit_message>
<xml_diff>
--- a/Documentation/HoferL-JournalPlanif-M5.xlsx
+++ b/Documentation/HoferL-JournalPlanif-M5.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
   <si>
     <t>date</t>
   </si>
@@ -286,6 +286,15 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;-- A jour avec la BDD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test de fonctionnement sur Windows, Linux et MacOS. Fonctionnel. Correction d'un dépendance sur Linux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de l'interface pour éditer les modules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implémentation des intéractions avec la BDD pour la gestion de module</t>
   </si>
   <si>
     <t>Phases</t>
@@ -1574,10 +1583,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3646,8 +3655,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E52">
-  <autoFilter ref="B2:E52"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E54">
+  <autoFilter ref="B2:E54"/>
   <tableColumns count="4">
     <tableColumn id="1" name="date" dataDxfId="0"/>
     <tableColumn id="2" name="Temps" dataDxfId="1"/>
@@ -4211,7 +4220,7 @@
       </c>
       <c r="I3" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.02412868632707775</v>
+        <v>2.3195876288659791e-002</v>
       </c>
       <c r="J3" s="12" t="str" cm="1">
         <f t="array" ref="J3:J9">_xlfn._xlws.FILTER(G3:G10,H3:H10&gt;0)</f>
@@ -4227,7 +4236,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>8</v>
@@ -4244,7 +4253,7 @@
       </c>
       <c r="I4" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.02412868632707775</v>
+        <v>2.3195876288659791e-002</v>
       </c>
       <c r="J4" s="4" t="str">
         <f/>
@@ -4277,7 +4286,7 @@
       </c>
       <c r="I5" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.072386058981233251</v>
+        <v>6.958762886597937e-002</v>
       </c>
       <c r="J5" s="4" t="str">
         <f/>
@@ -4293,7 +4302,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>8</v>
@@ -4310,7 +4319,7 @@
       </c>
       <c r="I6" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.13672922252010725</v>
+        <v>0.13144329896907214</v>
       </c>
       <c r="J6" s="4" t="str">
         <f/>
@@ -4326,7 +4335,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>8</v>
@@ -4343,7 +4352,7 @@
       </c>
       <c r="I7" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.30160857908847188</v>
+        <v>0.28994845360824739</v>
       </c>
       <c r="J7" s="4" t="str">
         <f/>
@@ -4372,11 +4381,11 @@
       </c>
       <c r="H8" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>53.500000000000007</v>
+        <v>58.500000000000014</v>
       </c>
       <c r="I8" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.4302949061662199</v>
+        <v>0.45231958762886604</v>
       </c>
       <c r="J8" s="4" t="str">
         <f/>
@@ -4384,7 +4393,7 @@
       </c>
       <c r="K8" s="13">
         <f/>
-        <v>53.500000000000007</v>
+        <v>58.500000000000014</v>
       </c>
     </row>
     <row r="9">
@@ -4409,7 +4418,7 @@
       </c>
       <c r="I9" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.010723860589812333</v>
+        <v>1.0309278350515462e-002</v>
       </c>
       <c r="J9" s="4" t="str">
         <f/>
@@ -4425,7 +4434,7 @@
         <v>22</v>
       </c>
       <c r="C10" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>12</v>
@@ -4452,7 +4461,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>12</v>
@@ -4465,7 +4474,7 @@
       </c>
       <c r="H11" s="10">
         <f>SUM(H3:H10)</f>
-        <v>124.33333333333333</v>
+        <v>129.33333333333334</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
@@ -4475,7 +4484,7 @@
         <v>22</v>
       </c>
       <c r="C12" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>10</v>
@@ -4490,7 +4499,7 @@
         <v>22</v>
       </c>
       <c r="C13" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>12</v>
@@ -4505,7 +4514,7 @@
         <v>29</v>
       </c>
       <c r="C14" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>12</v>
@@ -4561,7 +4570,7 @@
         <v>35</v>
       </c>
       <c r="C18" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>10</v>
@@ -4575,7 +4584,7 @@
         <v>37</v>
       </c>
       <c r="C19" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>12</v>
@@ -4589,7 +4598,7 @@
         <v>39</v>
       </c>
       <c r="C20" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>19</v>
@@ -4603,7 +4612,7 @@
         <v>39</v>
       </c>
       <c r="C21" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>15</v>
@@ -4631,7 +4640,7 @@
         <v>43</v>
       </c>
       <c r="C23" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>15</v>
@@ -4645,7 +4654,7 @@
         <v>45</v>
       </c>
       <c r="C24" s="6">
-        <v>0.0625</v>
+        <v>6.25e-002</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>15</v>
@@ -4687,7 +4696,7 @@
         <v>49</v>
       </c>
       <c r="C27" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>12</v>
@@ -4701,7 +4710,7 @@
         <v>52</v>
       </c>
       <c r="C28" s="6">
-        <v>0.0625</v>
+        <v>6.25e-002</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>15</v>
@@ -4743,7 +4752,7 @@
         <v>46087</v>
       </c>
       <c r="C31" s="6">
-        <v>0.020833333333333332</v>
+        <v>2.0833333333333332e-002</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>21</v>
@@ -4771,7 +4780,7 @@
         <v>46091</v>
       </c>
       <c r="C33" s="6">
-        <v>0.020833333333333332</v>
+        <v>2.0833333333333332e-002</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>12</v>
@@ -4799,7 +4808,7 @@
         <v>46091</v>
       </c>
       <c r="C35" s="6">
-        <v>0.020833333333333332</v>
+        <v>2.0833333333333332e-002</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>19</v>
@@ -4827,7 +4836,7 @@
         <v>46093</v>
       </c>
       <c r="C37" s="6">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>19</v>
@@ -4855,7 +4864,7 @@
         <v>46087</v>
       </c>
       <c r="C39" s="6">
-        <v>0.020833333333333332</v>
+        <v>2.0833333333333332e-002</v>
       </c>
       <c r="D39" s="7" t="s">
         <v>21</v>
@@ -4942,7 +4951,7 @@
         <v>46100</v>
       </c>
       <c r="C45" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D45" s="7" t="s">
         <v>8</v>
@@ -4956,7 +4965,7 @@
         <v>46100</v>
       </c>
       <c r="C46" s="6">
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>19</v>
@@ -4984,7 +4993,7 @@
         <v>46102</v>
       </c>
       <c r="C48" s="21">
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="D48" s="7" t="s">
         <v>8</v>
@@ -5043,26 +5052,42 @@
         <v>46104</v>
       </c>
       <c r="C52" s="21">
-        <v>0.013888888888888888</v>
-      </c>
-      <c r="D52" s="22" t="s">
+        <v>1.3888888888888888e-002</v>
+      </c>
+      <c r="D52" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E52" s="23" t="s">
-        <v>56</v>
+      <c r="E52" s="22" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="20"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="8"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="20"/>
-      <c r="C54" s="24"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="8"/>
+      <c r="B53" s="20">
+        <v>46117</v>
+      </c>
+      <c r="C53" s="21">
+        <v>0.125</v>
+      </c>
+      <c r="D53" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53" s="22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" ht="28.5">
+      <c r="B54" s="20">
+        <v>46118</v>
+      </c>
+      <c r="C54" s="21">
+        <v>8.3333333333333329e-002</v>
+      </c>
+      <c r="D54" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54" s="22" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="20"/>
@@ -5236,7 +5261,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{00DE0023-00B9-4D4C-941E-0023007B0050}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00D0007A-0025-4C9B-8357-00B900E50062}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$10</xm:f>
           </x14:formula1>
@@ -5269,7 +5294,7 @@
     </row>
     <row r="2">
       <c r="A2" s="25" t="str" cm="1">
-        <f t="array" ref="A2:A28">_xlfn.UNIQUE(Journal[date])</f>
+        <f t="array" ref="A2:A30">_xlfn.UNIQUE(Journal[date])</f>
         <v>20.01.2026</v>
       </c>
       <c r="B2" s="26">
@@ -5340,7 +5365,7 @@
       </c>
       <c r="B8" s="26">
         <f>SUMIF(Journal[date],SommeParJours!A8,Journal[Temps])</f>
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="C8"/>
     </row>
@@ -5351,7 +5376,7 @@
       </c>
       <c r="B9" s="26">
         <f>SUMIF(Journal[date],SommeParJours!A9,Journal[Temps])</f>
-        <v>0.041666666666666664</v>
+        <v>4.1666666666666664e-002</v>
       </c>
       <c r="C9"/>
     </row>
@@ -5373,7 +5398,7 @@
       </c>
       <c r="B11" s="26">
         <f>SUMIF(Journal[date],SommeParJours!A11,Journal[Temps])</f>
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="C11"/>
     </row>
@@ -5384,7 +5409,7 @@
       </c>
       <c r="B12" s="26">
         <f>SUMIF(Journal[date],SommeParJours!A12,Journal[Temps])</f>
-        <v>0.0625</v>
+        <v>6.25e-002</v>
       </c>
       <c r="C12"/>
     </row>
@@ -5461,7 +5486,7 @@
       </c>
       <c r="B19" s="26">
         <f>SUMIF(Journal[date],SommeParJours!A19,Journal[Temps])</f>
-        <v>0.083333333333333329</v>
+        <v>8.3333333333333329e-002</v>
       </c>
       <c r="C19"/>
     </row>
@@ -5567,21 +5592,27 @@
       </c>
       <c r="C28" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A28,Journal[Temps])</f>
-        <v>0.013888888888888888</v>
+        <v>1.3888888888888888e-002</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="25"/>
+      <c r="A29" s="25">
+        <f/>
+        <v>46117</v>
+      </c>
       <c r="C29" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A29,Journal[Temps])</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="25"/>
+      <c r="A30" s="25">
+        <f/>
+        <v>46118</v>
+      </c>
       <c r="C30" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A30,Journal[Temps])</f>
-        <v>0</v>
+        <v>8.3333333333333329e-002</v>
       </c>
     </row>
     <row r="31">
@@ -7028,16 +7059,16 @@
   <sheetData>
     <row r="1" s="32" customFormat="1" ht="66.599999999999994" customHeight="1">
       <c r="B1" s="33" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C1" s="34" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D1" s="35" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F1" s="36" t="s">
         <v>11</v>
@@ -7046,7 +7077,7 @@
         <v>17</v>
       </c>
       <c r="H1" s="38" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I1" s="35" t="s">
         <v>22</v>
@@ -7055,85 +7086,85 @@
         <v>37</v>
       </c>
       <c r="K1" s="35" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="L1" s="39" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="M1" s="35" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="N1" s="37" t="s">
         <v>47</v>
       </c>
       <c r="O1" s="38" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="P1" s="35" t="s">
         <v>49</v>
       </c>
       <c r="Q1" s="35" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="R1" s="35" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="S1" s="35" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="T1" s="35" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="U1" s="35" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="W1" s="40" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="X1" s="35" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="Y1" s="35" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AA1" s="41" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="AB1" s="42" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="AC1" s="42" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AD1" s="39" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="AE1" s="43" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="AF1" s="44" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="AG1" s="45" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="AH1" s="45" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AI1" s="45" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="AJ1" s="45" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="AK1" s="42" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="AL1" s="46"/>
       <c r="AM1" s="46"/>
@@ -7229,7 +7260,7 @@
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="47"/>
       <c r="C4" s="48" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D4" s="49"/>
       <c r="E4" s="49"/>
@@ -7385,7 +7416,7 @@
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="47"/>
       <c r="C8" s="48" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D8" s="63"/>
       <c r="E8" s="63"/>
@@ -7463,7 +7494,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="47"/>
       <c r="C10" s="48" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D10" s="49"/>
       <c r="E10" s="49"/>
@@ -7541,7 +7572,7 @@
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="47"/>
       <c r="C12" s="48" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D12" s="49"/>
       <c r="E12" s="49"/>
@@ -7618,10 +7649,10 @@
     </row>
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="65" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C14" s="66" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D14" s="63"/>
       <c r="E14" s="63"/>
@@ -7699,7 +7730,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="65"/>
       <c r="C16" s="66" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D16" s="63"/>
       <c r="E16" s="63"/>
@@ -7774,13 +7805,13 @@
       <c r="AJ17" s="68"/>
       <c r="AK17" s="68"/>
       <c r="AN17" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="65"/>
       <c r="C18" s="66" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D18" s="63"/>
       <c r="E18" s="63"/>
@@ -7858,7 +7889,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="65"/>
       <c r="C20" s="66" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D20" s="68"/>
       <c r="E20" s="68"/>
@@ -7936,7 +7967,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="65"/>
       <c r="C22" s="66" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D22" s="68"/>
       <c r="E22" s="68"/>
@@ -8014,7 +8045,7 @@
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="65"/>
       <c r="C24" s="66" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D24" s="68"/>
       <c r="E24" s="68"/>
@@ -8091,10 +8122,10 @@
     </row>
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="47" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C26" s="48" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D26" s="49"/>
       <c r="E26" s="49"/>
@@ -8172,7 +8203,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="47"/>
       <c r="C28" s="48" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D28" s="49"/>
       <c r="E28" s="49"/>
@@ -8250,7 +8281,7 @@
     <row r="30" ht="12" customHeight="1">
       <c r="B30" s="47"/>
       <c r="C30" s="48" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D30" s="49"/>
       <c r="E30" s="49"/>
@@ -8328,7 +8359,7 @@
     <row r="32" ht="12" customHeight="1">
       <c r="B32" s="47"/>
       <c r="C32" s="48" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D32" s="49"/>
       <c r="E32" s="49"/>
@@ -8405,10 +8436,10 @@
     </row>
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="65" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C34" s="74" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D34" s="68"/>
       <c r="E34" s="68"/>
@@ -8486,7 +8517,7 @@
     <row r="36" ht="12" customHeight="1">
       <c r="B36" s="65"/>
       <c r="C36" s="74" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D36" s="68"/>
       <c r="E36" s="68"/>
@@ -8564,7 +8595,7 @@
     <row r="38" ht="12" customHeight="1">
       <c r="B38" s="65"/>
       <c r="C38" s="74" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D38" s="68"/>
       <c r="E38" s="68"/>
@@ -8642,7 +8673,7 @@
     <row r="40" ht="12" customHeight="1">
       <c r="B40" s="65"/>
       <c r="C40" s="74" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D40" s="68"/>
       <c r="E40" s="68"/>
@@ -8722,7 +8753,7 @@
         <v>21</v>
       </c>
       <c r="C42" s="77" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D42" s="49"/>
       <c r="E42" s="49"/>
@@ -8800,7 +8831,7 @@
     <row r="44" ht="12" customHeight="1">
       <c r="B44" s="47"/>
       <c r="C44" s="77" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D44" s="49"/>
       <c r="E44" s="49"/>
@@ -8877,7 +8908,7 @@
     </row>
     <row r="46" ht="12" customHeight="1">
       <c r="B46" s="65" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C46" s="66" t="s">
         <v>24</v>
@@ -8955,14 +8986,14 @@
       <c r="AJ47" s="68"/>
       <c r="AK47" s="68"/>
       <c r="AN47" s="78" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="AO47" s="63"/>
     </row>
     <row r="48" ht="12" customHeight="1">
       <c r="B48" s="65"/>
       <c r="C48" s="66" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D48" s="68"/>
       <c r="E48" s="68"/>
@@ -8999,7 +9030,7 @@
       <c r="AJ48" s="68"/>
       <c r="AK48" s="79"/>
       <c r="AN48" s="78" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="AO48" s="62"/>
     </row>
@@ -9041,7 +9072,7 @@
       <c r="AJ49" s="68"/>
       <c r="AK49" s="68"/>
       <c r="AN49" s="78" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AO49" s="58"/>
     </row>
@@ -9110,37 +9141,37 @@
     </row>
     <row r="2" ht="56.399999999999999" customHeight="1">
       <c r="B2" s="81" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D2" s="83" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E2" s="84" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F2" s="85" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G2" s="85"/>
       <c r="H2" s="85"/>
       <c r="I2" s="84"/>
       <c r="J2" s="85" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="K2" s="85"/>
       <c r="L2" s="85"/>
       <c r="M2" s="84"/>
       <c r="N2" s="85" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="O2" s="85"/>
       <c r="P2" s="85"/>
       <c r="Q2" s="84"/>
       <c r="R2" s="85" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="S2" s="86"/>
       <c r="AD2" s="29"/>
@@ -9149,7 +9180,7 @@
       <c r="B3" s="87"/>
       <c r="C3" s="88"/>
       <c r="D3" s="89" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E3" s="90">
         <v>4</v>
@@ -9197,15 +9228,15 @@
         <v>2</v>
       </c>
       <c r="U3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="94" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D4" s="95"/>
       <c r="E4" s="96"/>
@@ -9224,7 +9255,7 @@
       <c r="R4" s="99"/>
       <c r="S4" s="100"/>
       <c r="U4" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -9250,7 +9281,7 @@
     <row r="6" ht="12" customHeight="1">
       <c r="B6" s="94"/>
       <c r="C6" s="109" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D6" s="110"/>
       <c r="E6" s="111"/>
@@ -9269,7 +9300,7 @@
       <c r="R6" s="115"/>
       <c r="S6" s="116"/>
       <c r="U6" s="117" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="V6" s="117"/>
     </row>
@@ -9293,13 +9324,13 @@
       <c r="R7" s="107"/>
       <c r="S7" s="108"/>
       <c r="U7" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="94"/>
       <c r="C8" s="109" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D8" s="110"/>
       <c r="E8" s="111"/>
@@ -9318,7 +9349,7 @@
       <c r="R8" s="115"/>
       <c r="S8" s="116"/>
       <c r="U8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -9344,7 +9375,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="94"/>
       <c r="C10" s="109" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D10" s="110"/>
       <c r="E10" s="111"/>
@@ -9385,10 +9416,10 @@
     </row>
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="81" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C12" s="82" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D12" s="95"/>
       <c r="E12" s="96"/>
@@ -9430,7 +9461,7 @@
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="94"/>
       <c r="C14" s="109" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D14" s="128"/>
       <c r="E14" s="111"/>
@@ -9472,7 +9503,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="94"/>
       <c r="C16" s="109" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D16" s="110"/>
       <c r="E16" s="111"/>
@@ -9513,10 +9544,10 @@
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="83" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C18" s="82" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D18" s="95"/>
       <c r="E18" s="96"/>
@@ -9558,7 +9589,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="94"/>
       <c r="C20" s="109" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D20" s="110"/>
       <c r="E20" s="111"/>
@@ -9600,7 +9631,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="94"/>
       <c r="C22" s="109" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D22" s="110"/>
       <c r="E22" s="111"/>
@@ -9641,10 +9672,10 @@
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="83" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C24" s="82" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D24" s="95"/>
       <c r="E24" s="96"/>
@@ -9686,7 +9717,7 @@
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="94"/>
       <c r="C26" s="109" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D26" s="110"/>
       <c r="E26" s="111"/>
@@ -9728,7 +9759,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="94"/>
       <c r="C28" s="109" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D28" s="110"/>
       <c r="E28" s="111"/>
@@ -9772,7 +9803,7 @@
         <v>12</v>
       </c>
       <c r="C30" s="141" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D30" s="95"/>
       <c r="E30" s="142"/>
@@ -9856,7 +9887,7 @@
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="147"/>
       <c r="C34" s="101" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D34" s="133"/>
       <c r="E34" s="161"/>
@@ -9876,7 +9907,7 @@
       <c r="S34" s="165"/>
       <c r="U34" s="166"/>
       <c r="V34" s="167" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" ht="13.800000000000001" customHeight="1">
@@ -9900,7 +9931,7 @@
       <c r="S35" s="125"/>
       <c r="U35" s="174"/>
       <c r="V35" s="175" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise a jour du suivit
Journal de travail + version logiciels
</commit_message>
<xml_diff>
--- a/Documentation/HoferL-JournalPlanif-M5.xlsx
+++ b/Documentation/HoferL-JournalPlanif-M5.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="1" state="visible" r:id="rId4"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="172">
   <si>
     <t>date</t>
   </si>
@@ -285,16 +285,25 @@
     <t xml:space="preserve">Finalisation du PoC. Très concluant, fonctionnel et fluide. Merge de la branche PDF -&gt; Main.</t>
   </si>
   <si>
+    <t xml:space="preserve">Test de fonctionnement sur Windows, Linux et MacOS. Fonctionnel. Correction d'un dépendance sur Linux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de l'interface pour éditer les modules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implémentation des intéractions avec la BDD pour la gestion de module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lecture de la mise a jour d'Avalonia 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migration avalonia 11.3.13 vers 12.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction de fonctionnement + Optimisation et suppression de mem leak</t>
+  </si>
+  <si>
     <t xml:space="preserve">&lt;-- A jour avec la BDD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test de fonctionnement sur Windows, Linux et MacOS. Fonctionnel. Correction d'un dépendance sur Linux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ajout de l'interface pour éditer les modules</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implémentation des intéractions avec la BDD pour la gestion de module</t>
   </si>
   <si>
     <t>Phases</t>
@@ -2198,7 +2207,7 @@
                   <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>17</c:v>
@@ -2207,7 +2216,7 @@
                   <c:v>37.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>53.50000000000001</c:v>
+                  <c:v>63.000000000000014</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2434,9 +2443,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>SommeParJours!$A$2:$A$27</c:f>
+              <c:f>SommeParJours!$A$2:$A$32</c:f>
               <c:strCache>
-                <c:ptCount val="26"/>
+                <c:ptCount val="31"/>
                 <c:pt idx="0">
                   <c:v>20.01.2026</c:v>
                 </c:pt>
@@ -2515,15 +2524,30 @@
                 <c:pt idx="25">
                   <c:v>3/22/2026</c:v>
                 </c:pt>
+                <c:pt idx="26">
+                  <c:v>3/23/2026</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4/5/2026</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>4/6/2026</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>4/7/2026</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>4/10/2026</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>SommeParJours!$B$2:$B$27</c:f>
+              <c:f>SommeParJours!$B$2:$B$32</c:f>
               <c:numCache>
                 <c:formatCode>h:mm;@</c:formatCode>
-                <c:ptCount val="26"/>
+                <c:ptCount val="31"/>
                 <c:pt idx="0">
                   <c:v>0.16666666666666666</c:v>
                 </c:pt>
@@ -2601,6 +2625,21 @@
                 </c:pt>
                 <c:pt idx="25">
                   <c:v>0.375</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.013888888888888888</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.125</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.08333333333333333</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.08333333333333333</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3655,8 +3694,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E54">
-  <autoFilter ref="B2:E54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Journal" ref="B2:E57">
+  <autoFilter ref="B2:E57"/>
   <tableColumns count="4">
     <tableColumn id="1" name="date" dataDxfId="0"/>
     <tableColumn id="2" name="Temps" dataDxfId="1"/>
@@ -4220,7 +4259,7 @@
       </c>
       <c r="I3" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>2.3195876288659791e-002</v>
+        <v>2.2332506203473945e-002</v>
       </c>
       <c r="J3" s="12" t="str" cm="1">
         <f t="array" ref="J3:J9">_xlfn._xlws.FILTER(G3:G10,H3:H10&gt;0)</f>
@@ -4253,7 +4292,7 @@
       </c>
       <c r="I4" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>2.3195876288659791e-002</v>
+        <v>2.2332506203473945e-002</v>
       </c>
       <c r="J4" s="4" t="str">
         <f/>
@@ -4282,11 +4321,11 @@
       </c>
       <c r="H5" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="I5" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>6.958762886597937e-002</v>
+        <v>7.0719602977667495e-002</v>
       </c>
       <c r="J5" s="4" t="str">
         <f/>
@@ -4294,7 +4333,7 @@
       </c>
       <c r="K5" s="13">
         <f/>
-        <v>9</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="6">
@@ -4319,7 +4358,7 @@
       </c>
       <c r="I6" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.13144329896907214</v>
+        <v>0.12655086848635236</v>
       </c>
       <c r="J6" s="4" t="str">
         <f/>
@@ -4352,7 +4391,7 @@
       </c>
       <c r="I7" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.28994845360824739</v>
+        <v>0.27915632754342429</v>
       </c>
       <c r="J7" s="4" t="str">
         <f/>
@@ -4381,11 +4420,11 @@
       </c>
       <c r="H8" s="10">
         <f>SUMIF(Journal[type de travail],types[[#This Row],[type de travail]],Journal[Temps])*24</f>
-        <v>58.500000000000014</v>
+        <v>63.000000000000014</v>
       </c>
       <c r="I8" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>0.45231958762886604</v>
+        <v>0.46898263027295295</v>
       </c>
       <c r="J8" s="4" t="str">
         <f/>
@@ -4393,7 +4432,7 @@
       </c>
       <c r="K8" s="13">
         <f/>
-        <v>58.500000000000014</v>
+        <v>63.000000000000014</v>
       </c>
     </row>
     <row r="9">
@@ -4418,7 +4457,7 @@
       </c>
       <c r="I9" s="11">
         <f>types[[#This Row],[somme]]/$H$11</f>
-        <v>1.0309278350515462e-002</v>
+        <v>9.9255583126550851e-003</v>
       </c>
       <c r="J9" s="4" t="str">
         <f/>
@@ -4474,7 +4513,7 @@
       </c>
       <c r="H11" s="10">
         <f>SUM(H3:H10)</f>
-        <v>129.33333333333334</v>
+        <v>134.33333333333334</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
@@ -5043,9 +5082,6 @@
       <c r="E51" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G51" t="s">
-        <v>76</v>
-      </c>
     </row>
     <row r="52" ht="28.5">
       <c r="B52" s="20">
@@ -5058,7 +5094,7 @@
         <v>21</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="53">
@@ -5068,11 +5104,11 @@
       <c r="C53" s="21">
         <v>0.125</v>
       </c>
-      <c r="D53" s="23" t="s">
+      <c r="D53" s="7" t="s">
         <v>19</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="54" ht="28.5">
@@ -5082,30 +5118,57 @@
       <c r="C54" s="21">
         <v>8.3333333333333329e-002</v>
       </c>
-      <c r="D54" s="23" t="s">
+      <c r="D54" s="7" t="s">
         <v>19</v>
       </c>
       <c r="E54" s="22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="20">
+        <v>46119</v>
+      </c>
+      <c r="C55" s="21">
+        <v>2.0833333333333332e-002</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="22" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" s="20"/>
-      <c r="C55" s="24"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="8"/>
-    </row>
     <row r="56">
-      <c r="B56" s="20"/>
-      <c r="C56" s="24"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="8"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="20"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="8"/>
+      <c r="B56" s="20">
+        <v>46119</v>
+      </c>
+      <c r="C56" s="21">
+        <v>6.25e-002</v>
+      </c>
+      <c r="D56" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E56" s="22" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" ht="28.5">
+      <c r="B57" s="20">
+        <v>46122</v>
+      </c>
+      <c r="C57" s="21">
+        <v>0.125</v>
+      </c>
+      <c r="D57" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="G57" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="20"/>
@@ -5261,7 +5324,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{00D0007A-0025-4C9B-8357-00B900E50062}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{001E0023-0082-40B6-BF21-00E4006D006F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$G$3:$G$10</xm:f>
           </x14:formula1>
@@ -5294,7 +5357,7 @@
     </row>
     <row r="2">
       <c r="A2" s="25" t="str" cm="1">
-        <f t="array" ref="A2:A30">_xlfn.UNIQUE(Journal[date])</f>
+        <f t="array" ref="A2:A32">_xlfn.UNIQUE(Journal[date])</f>
         <v>20.01.2026</v>
       </c>
       <c r="B2" s="26">
@@ -5590,6 +5653,10 @@
         <f/>
         <v>46104</v>
       </c>
+      <c r="B28" s="26">
+        <f>SUMIF(Journal[date],SommeParJours!A28,Journal[Temps])</f>
+        <v>1.3888888888888888e-002</v>
+      </c>
       <c r="C28" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A28,Journal[Temps])</f>
         <v>1.3888888888888888e-002</v>
@@ -5600,6 +5667,10 @@
         <f/>
         <v>46117</v>
       </c>
+      <c r="B29" s="26">
+        <f>SUMIF(Journal[date],SommeParJours!A29,Journal[Temps])</f>
+        <v>0.125</v>
+      </c>
       <c r="C29" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A29,Journal[Temps])</f>
         <v>0.125</v>
@@ -5610,23 +5681,41 @@
         <f/>
         <v>46118</v>
       </c>
+      <c r="B30" s="26">
+        <f>SUMIF(Journal[date],SommeParJours!A30,Journal[Temps])</f>
+        <v>8.3333333333333329e-002</v>
+      </c>
       <c r="C30" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A30,Journal[Temps])</f>
         <v>8.3333333333333329e-002</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="25"/>
+      <c r="A31" s="25">
+        <f/>
+        <v>46119</v>
+      </c>
+      <c r="B31" s="26">
+        <f>SUMIF(Journal[date],SommeParJours!A31,Journal[Temps])</f>
+        <v>8.3333333333333329e-002</v>
+      </c>
       <c r="C31" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A31,Journal[Temps])</f>
-        <v>0</v>
+        <v>8.3333333333333329e-002</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="25"/>
+      <c r="A32" s="25">
+        <f/>
+        <v>46122</v>
+      </c>
+      <c r="B32" s="26">
+        <f>SUMIF(Journal[date],SommeParJours!A32,Journal[Temps])</f>
+        <v>0.125</v>
+      </c>
       <c r="C32" s="28">
         <f>SUMIF(Journal[date],SommeParJours!A32,Journal[Temps])</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="33">
@@ -7059,16 +7148,16 @@
   <sheetData>
     <row r="1" s="32" customFormat="1" ht="66.599999999999994" customHeight="1">
       <c r="B1" s="33" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C1" s="34" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D1" s="35" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F1" s="36" t="s">
         <v>11</v>
@@ -7077,7 +7166,7 @@
         <v>17</v>
       </c>
       <c r="H1" s="38" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="I1" s="35" t="s">
         <v>22</v>
@@ -7086,85 +7175,85 @@
         <v>37</v>
       </c>
       <c r="K1" s="35" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="L1" s="39" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="M1" s="35" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="N1" s="37" t="s">
         <v>47</v>
       </c>
       <c r="O1" s="38" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="P1" s="35" t="s">
         <v>49</v>
       </c>
       <c r="Q1" s="35" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="R1" s="35" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="S1" s="35" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="T1" s="35" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="U1" s="35" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="V1" s="37" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="W1" s="40" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="X1" s="35" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="Y1" s="35" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="Z1" s="37" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="AA1" s="41" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="AB1" s="42" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="AC1" s="42" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="AD1" s="39" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="AE1" s="43" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="AF1" s="44" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="AG1" s="45" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="AH1" s="45" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="AI1" s="45" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="AJ1" s="45" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="AK1" s="42" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="AL1" s="46"/>
       <c r="AM1" s="46"/>
@@ -7260,7 +7349,7 @@
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="47"/>
       <c r="C4" s="48" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D4" s="49"/>
       <c r="E4" s="49"/>
@@ -7416,7 +7505,7 @@
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="47"/>
       <c r="C8" s="48" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D8" s="63"/>
       <c r="E8" s="63"/>
@@ -7494,7 +7583,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="47"/>
       <c r="C10" s="48" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D10" s="49"/>
       <c r="E10" s="49"/>
@@ -7572,7 +7661,7 @@
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="47"/>
       <c r="C12" s="48" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D12" s="49"/>
       <c r="E12" s="49"/>
@@ -7649,10 +7738,10 @@
     </row>
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="65" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C14" s="66" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D14" s="63"/>
       <c r="E14" s="63"/>
@@ -7730,7 +7819,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="65"/>
       <c r="C16" s="66" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D16" s="63"/>
       <c r="E16" s="63"/>
@@ -7805,13 +7894,13 @@
       <c r="AJ17" s="68"/>
       <c r="AK17" s="68"/>
       <c r="AN17" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="65"/>
       <c r="C18" s="66" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D18" s="63"/>
       <c r="E18" s="63"/>
@@ -7889,7 +7978,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="65"/>
       <c r="C20" s="66" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D20" s="68"/>
       <c r="E20" s="68"/>
@@ -7967,7 +8056,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="65"/>
       <c r="C22" s="66" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D22" s="68"/>
       <c r="E22" s="68"/>
@@ -8045,7 +8134,7 @@
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="65"/>
       <c r="C24" s="66" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D24" s="68"/>
       <c r="E24" s="68"/>
@@ -8122,10 +8211,10 @@
     </row>
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="47" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C26" s="48" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D26" s="49"/>
       <c r="E26" s="49"/>
@@ -8203,7 +8292,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="47"/>
       <c r="C28" s="48" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D28" s="49"/>
       <c r="E28" s="49"/>
@@ -8281,7 +8370,7 @@
     <row r="30" ht="12" customHeight="1">
       <c r="B30" s="47"/>
       <c r="C30" s="48" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D30" s="49"/>
       <c r="E30" s="49"/>
@@ -8359,7 +8448,7 @@
     <row r="32" ht="12" customHeight="1">
       <c r="B32" s="47"/>
       <c r="C32" s="48" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D32" s="49"/>
       <c r="E32" s="49"/>
@@ -8436,10 +8525,10 @@
     </row>
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="65" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C34" s="74" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D34" s="68"/>
       <c r="E34" s="68"/>
@@ -8517,7 +8606,7 @@
     <row r="36" ht="12" customHeight="1">
       <c r="B36" s="65"/>
       <c r="C36" s="74" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D36" s="68"/>
       <c r="E36" s="68"/>
@@ -8595,7 +8684,7 @@
     <row r="38" ht="12" customHeight="1">
       <c r="B38" s="65"/>
       <c r="C38" s="74" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D38" s="68"/>
       <c r="E38" s="68"/>
@@ -8673,7 +8762,7 @@
     <row r="40" ht="12" customHeight="1">
       <c r="B40" s="65"/>
       <c r="C40" s="74" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D40" s="68"/>
       <c r="E40" s="68"/>
@@ -8753,7 +8842,7 @@
         <v>21</v>
       </c>
       <c r="C42" s="77" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D42" s="49"/>
       <c r="E42" s="49"/>
@@ -8831,7 +8920,7 @@
     <row r="44" ht="12" customHeight="1">
       <c r="B44" s="47"/>
       <c r="C44" s="77" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D44" s="49"/>
       <c r="E44" s="49"/>
@@ -8908,7 +8997,7 @@
     </row>
     <row r="46" ht="12" customHeight="1">
       <c r="B46" s="65" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C46" s="66" t="s">
         <v>24</v>
@@ -8986,14 +9075,14 @@
       <c r="AJ47" s="68"/>
       <c r="AK47" s="68"/>
       <c r="AN47" s="78" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AO47" s="63"/>
     </row>
     <row r="48" ht="12" customHeight="1">
       <c r="B48" s="65"/>
       <c r="C48" s="66" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D48" s="68"/>
       <c r="E48" s="68"/>
@@ -9030,7 +9119,7 @@
       <c r="AJ48" s="68"/>
       <c r="AK48" s="79"/>
       <c r="AN48" s="78" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AO48" s="62"/>
     </row>
@@ -9072,7 +9161,7 @@
       <c r="AJ49" s="68"/>
       <c r="AK49" s="68"/>
       <c r="AN49" s="78" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AO49" s="58"/>
     </row>
@@ -9141,37 +9230,37 @@
     </row>
     <row r="2" ht="56.399999999999999" customHeight="1">
       <c r="B2" s="81" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D2" s="83" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E2" s="84" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F2" s="85" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="G2" s="85"/>
       <c r="H2" s="85"/>
       <c r="I2" s="84"/>
       <c r="J2" s="85" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="K2" s="85"/>
       <c r="L2" s="85"/>
       <c r="M2" s="84"/>
       <c r="N2" s="85" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="O2" s="85"/>
       <c r="P2" s="85"/>
       <c r="Q2" s="84"/>
       <c r="R2" s="85" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="S2" s="86"/>
       <c r="AD2" s="29"/>
@@ -9180,7 +9269,7 @@
       <c r="B3" s="87"/>
       <c r="C3" s="88"/>
       <c r="D3" s="89" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E3" s="90">
         <v>4</v>
@@ -9228,15 +9317,15 @@
         <v>2</v>
       </c>
       <c r="U3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" ht="12" customHeight="1">
       <c r="B4" s="94" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D4" s="95"/>
       <c r="E4" s="96"/>
@@ -9255,7 +9344,7 @@
       <c r="R4" s="99"/>
       <c r="S4" s="100"/>
       <c r="U4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1">
@@ -9281,7 +9370,7 @@
     <row r="6" ht="12" customHeight="1">
       <c r="B6" s="94"/>
       <c r="C6" s="109" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D6" s="110"/>
       <c r="E6" s="111"/>
@@ -9300,7 +9389,7 @@
       <c r="R6" s="115"/>
       <c r="S6" s="116"/>
       <c r="U6" s="117" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="V6" s="117"/>
     </row>
@@ -9324,13 +9413,13 @@
       <c r="R7" s="107"/>
       <c r="S7" s="108"/>
       <c r="U7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" ht="12" customHeight="1">
       <c r="B8" s="94"/>
       <c r="C8" s="109" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D8" s="110"/>
       <c r="E8" s="111"/>
@@ -9349,7 +9438,7 @@
       <c r="R8" s="115"/>
       <c r="S8" s="116"/>
       <c r="U8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -9375,7 +9464,7 @@
     <row r="10" ht="12" customHeight="1">
       <c r="B10" s="94"/>
       <c r="C10" s="109" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D10" s="110"/>
       <c r="E10" s="111"/>
@@ -9416,10 +9505,10 @@
     </row>
     <row r="12" ht="12" customHeight="1">
       <c r="B12" s="81" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C12" s="82" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D12" s="95"/>
       <c r="E12" s="96"/>
@@ -9461,7 +9550,7 @@
     <row r="14" ht="12" customHeight="1">
       <c r="B14" s="94"/>
       <c r="C14" s="109" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D14" s="128"/>
       <c r="E14" s="111"/>
@@ -9503,7 +9592,7 @@
     <row r="16" ht="12" customHeight="1">
       <c r="B16" s="94"/>
       <c r="C16" s="109" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D16" s="110"/>
       <c r="E16" s="111"/>
@@ -9544,10 +9633,10 @@
     </row>
     <row r="18" ht="12" customHeight="1">
       <c r="B18" s="83" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C18" s="82" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D18" s="95"/>
       <c r="E18" s="96"/>
@@ -9589,7 +9678,7 @@
     <row r="20" ht="12" customHeight="1">
       <c r="B20" s="94"/>
       <c r="C20" s="109" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D20" s="110"/>
       <c r="E20" s="111"/>
@@ -9631,7 +9720,7 @@
     <row r="22" ht="12" customHeight="1">
       <c r="B22" s="94"/>
       <c r="C22" s="109" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D22" s="110"/>
       <c r="E22" s="111"/>
@@ -9672,10 +9761,10 @@
     </row>
     <row r="24" ht="12" customHeight="1">
       <c r="B24" s="83" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C24" s="82" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D24" s="95"/>
       <c r="E24" s="96"/>
@@ -9717,7 +9806,7 @@
     <row r="26" ht="12" customHeight="1">
       <c r="B26" s="94"/>
       <c r="C26" s="109" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D26" s="110"/>
       <c r="E26" s="111"/>
@@ -9759,7 +9848,7 @@
     <row r="28" ht="12" customHeight="1">
       <c r="B28" s="94"/>
       <c r="C28" s="109" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D28" s="110"/>
       <c r="E28" s="111"/>
@@ -9803,7 +9892,7 @@
         <v>12</v>
       </c>
       <c r="C30" s="141" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D30" s="95"/>
       <c r="E30" s="142"/>
@@ -9887,7 +9976,7 @@
     <row r="34" ht="12" customHeight="1">
       <c r="B34" s="147"/>
       <c r="C34" s="101" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D34" s="133"/>
       <c r="E34" s="161"/>
@@ -9907,7 +9996,7 @@
       <c r="S34" s="165"/>
       <c r="U34" s="166"/>
       <c r="V34" s="167" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" ht="13.800000000000001" customHeight="1">
@@ -9931,7 +10020,7 @@
       <c r="S35" s="125"/>
       <c r="U35" s="174"/>
       <c r="V35" s="175" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>